<commit_message>
Added pre-race data for Baku
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -3223,6 +3223,15 @@
   </si>
   <si>
     <t>19-5</t>
+  </si>
+  <si>
+    <t>13-10</t>
+  </si>
+  <si>
+    <t>30-1</t>
+  </si>
+  <si>
+    <t>175-1</t>
   </si>
 </sst>
 </file>
@@ -10278,6 +10287,446 @@
         <v>106</v>
       </c>
     </row>
+    <row r="310">
+      <c r="A310" t="s">
+        <v>955</v>
+      </c>
+      <c r="B310" t="s">
+        <v>956</v>
+      </c>
+      <c r="C310">
+        <v>2026</v>
+      </c>
+      <c r="D310" s="0">
+        <v>15</v>
+      </c>
+      <c r="E310" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F310" s="10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="s">
+        <v>960</v>
+      </c>
+      <c r="B311" t="s">
+        <v>961</v>
+      </c>
+      <c r="C311">
+        <v>2026</v>
+      </c>
+      <c r="D311" s="0">
+        <v>15</v>
+      </c>
+      <c r="E311" s="10" t="s">
+        <v>1071</v>
+      </c>
+      <c r="F311" s="10" t="s">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="s">
+        <v>965</v>
+      </c>
+      <c r="B312" t="s">
+        <v>966</v>
+      </c>
+      <c r="C312">
+        <v>2026</v>
+      </c>
+      <c r="D312" s="0">
+        <v>15</v>
+      </c>
+      <c r="E312" s="10" t="s">
+        <v>988</v>
+      </c>
+      <c r="F312" s="10" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="s">
+        <v>970</v>
+      </c>
+      <c r="B313" t="s">
+        <v>971</v>
+      </c>
+      <c r="C313">
+        <v>2026</v>
+      </c>
+      <c r="D313" s="0">
+        <v>15</v>
+      </c>
+      <c r="E313" s="10" t="s">
+        <v>1070</v>
+      </c>
+      <c r="F313" s="10" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="s">
+        <v>975</v>
+      </c>
+      <c r="B314" t="s">
+        <v>976</v>
+      </c>
+      <c r="C314">
+        <v>2026</v>
+      </c>
+      <c r="D314" s="0">
+        <v>15</v>
+      </c>
+      <c r="E314" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F314" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="s">
+        <v>980</v>
+      </c>
+      <c r="B315" t="s">
+        <v>981</v>
+      </c>
+      <c r="C315">
+        <v>2026</v>
+      </c>
+      <c r="D315" s="0">
+        <v>15</v>
+      </c>
+      <c r="E315" s="10" t="s">
+        <v>675</v>
+      </c>
+      <c r="F315" s="10" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="s">
+        <v>985</v>
+      </c>
+      <c r="B316" t="s">
+        <v>986</v>
+      </c>
+      <c r="C316">
+        <v>2026</v>
+      </c>
+      <c r="D316" s="0">
+        <v>15</v>
+      </c>
+      <c r="E316" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="F316" s="10" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="s">
+        <v>990</v>
+      </c>
+      <c r="B317" t="s">
+        <v>991</v>
+      </c>
+      <c r="C317">
+        <v>2026</v>
+      </c>
+      <c r="D317" s="0">
+        <v>15</v>
+      </c>
+      <c r="E317" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="F317" s="10" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="s">
+        <v>995</v>
+      </c>
+      <c r="B318" t="s">
+        <v>996</v>
+      </c>
+      <c r="C318">
+        <v>2026</v>
+      </c>
+      <c r="D318" s="0">
+        <v>15</v>
+      </c>
+      <c r="E318" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="F318" s="10" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B319" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C319">
+        <v>2026</v>
+      </c>
+      <c r="D319" s="0">
+        <v>15</v>
+      </c>
+      <c r="E319" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="F319" s="10" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B320" t="s">
+        <v>1006</v>
+      </c>
+      <c r="C320">
+        <v>2026</v>
+      </c>
+      <c r="D320" s="0">
+        <v>15</v>
+      </c>
+      <c r="E320" s="10" t="s">
+        <v>1067</v>
+      </c>
+      <c r="F320" s="10" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B321" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C321">
+        <v>2026</v>
+      </c>
+      <c r="D321" s="0">
+        <v>15</v>
+      </c>
+      <c r="E321" s="10" t="s">
+        <v>897</v>
+      </c>
+      <c r="F321" s="10" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B322" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C322">
+        <v>2026</v>
+      </c>
+      <c r="D322" s="0">
+        <v>15</v>
+      </c>
+      <c r="E322" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="F322" s="10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B323" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C323">
+        <v>2026</v>
+      </c>
+      <c r="D323" s="0">
+        <v>15</v>
+      </c>
+      <c r="E323" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="F323" s="10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B324" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C324">
+        <v>2026</v>
+      </c>
+      <c r="D324" s="0">
+        <v>15</v>
+      </c>
+      <c r="E324" s="10" t="s">
+        <v>897</v>
+      </c>
+      <c r="F324" s="10" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B325" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C325">
+        <v>2026</v>
+      </c>
+      <c r="D325" s="0">
+        <v>15</v>
+      </c>
+      <c r="E325" s="10" t="s">
+        <v>1067</v>
+      </c>
+      <c r="F325" s="10" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B326" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C326">
+        <v>2026</v>
+      </c>
+      <c r="D326" s="0">
+        <v>15</v>
+      </c>
+      <c r="E326" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F326" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B327" t="s">
+        <v>1041</v>
+      </c>
+      <c r="C327">
+        <v>2026</v>
+      </c>
+      <c r="D327" s="0">
+        <v>15</v>
+      </c>
+      <c r="E327" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F327" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B328" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C328">
+        <v>2026</v>
+      </c>
+      <c r="D328" s="0">
+        <v>15</v>
+      </c>
+      <c r="E328" s="10" t="s">
+        <v>1072</v>
+      </c>
+      <c r="F328" s="10" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B329" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C329">
+        <v>2026</v>
+      </c>
+      <c r="D329" s="0">
+        <v>15</v>
+      </c>
+      <c r="E329" s="10" t="s">
+        <v>897</v>
+      </c>
+      <c r="F329" s="10" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B330" t="s">
+        <v>1056</v>
+      </c>
+      <c r="C330">
+        <v>2026</v>
+      </c>
+      <c r="D330" s="0">
+        <v>15</v>
+      </c>
+      <c r="E330" s="10" t="s">
+        <v>345</v>
+      </c>
+      <c r="F330" s="10" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B331" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C331">
+        <v>2026</v>
+      </c>
+      <c r="D331" s="0">
+        <v>15</v>
+      </c>
+      <c r="E331" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="F331" s="10" t="s">
+        <v>193</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated stats and team selection for Malaysia
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -3232,6 +3232,12 @@
   </si>
   <si>
     <t>175-1</t>
+  </si>
+  <si>
+    <t>17-5</t>
+  </si>
+  <si>
+    <t>17-2</t>
   </si>
 </sst>
 </file>
@@ -10727,6 +10733,446 @@
         <v>193</v>
       </c>
     </row>
+    <row r="332">
+      <c r="A332" t="s">
+        <v>955</v>
+      </c>
+      <c r="B332" t="s">
+        <v>956</v>
+      </c>
+      <c r="C332">
+        <v>2026</v>
+      </c>
+      <c r="D332" s="0">
+        <v>16</v>
+      </c>
+      <c r="E332" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F332" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="s">
+        <v>960</v>
+      </c>
+      <c r="B333" t="s">
+        <v>961</v>
+      </c>
+      <c r="C333">
+        <v>2026</v>
+      </c>
+      <c r="D333" s="0">
+        <v>16</v>
+      </c>
+      <c r="E333" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="F333" s="10" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="s">
+        <v>965</v>
+      </c>
+      <c r="B334" t="s">
+        <v>966</v>
+      </c>
+      <c r="C334">
+        <v>2026</v>
+      </c>
+      <c r="D334" s="0">
+        <v>16</v>
+      </c>
+      <c r="E334" s="10" t="s">
+        <v>1073</v>
+      </c>
+      <c r="F334" s="10" t="s">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="s">
+        <v>970</v>
+      </c>
+      <c r="B335" t="s">
+        <v>971</v>
+      </c>
+      <c r="C335">
+        <v>2026</v>
+      </c>
+      <c r="D335" s="0">
+        <v>16</v>
+      </c>
+      <c r="E335" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="F335" s="10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="s">
+        <v>975</v>
+      </c>
+      <c r="B336" t="s">
+        <v>976</v>
+      </c>
+      <c r="C336">
+        <v>2026</v>
+      </c>
+      <c r="D336" s="0">
+        <v>16</v>
+      </c>
+      <c r="E336" s="10" t="s">
+        <v>1074</v>
+      </c>
+      <c r="F336" s="10" t="s">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="s">
+        <v>980</v>
+      </c>
+      <c r="B337" t="s">
+        <v>981</v>
+      </c>
+      <c r="C337">
+        <v>2026</v>
+      </c>
+      <c r="D337" s="0">
+        <v>16</v>
+      </c>
+      <c r="E337" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="F337" s="10" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="s">
+        <v>985</v>
+      </c>
+      <c r="B338" t="s">
+        <v>986</v>
+      </c>
+      <c r="C338">
+        <v>2026</v>
+      </c>
+      <c r="D338" s="0">
+        <v>16</v>
+      </c>
+      <c r="E338" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F338" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="s">
+        <v>990</v>
+      </c>
+      <c r="B339" t="s">
+        <v>991</v>
+      </c>
+      <c r="C339">
+        <v>2026</v>
+      </c>
+      <c r="D339" s="0">
+        <v>16</v>
+      </c>
+      <c r="E339" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F339" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="s">
+        <v>995</v>
+      </c>
+      <c r="B340" t="s">
+        <v>996</v>
+      </c>
+      <c r="C340">
+        <v>2026</v>
+      </c>
+      <c r="D340" s="0">
+        <v>16</v>
+      </c>
+      <c r="E340" s="10" t="s">
+        <v>1067</v>
+      </c>
+      <c r="F340" s="10" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B341" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C341">
+        <v>2026</v>
+      </c>
+      <c r="D341" s="0">
+        <v>16</v>
+      </c>
+      <c r="E341" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F341" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B342" t="s">
+        <v>1006</v>
+      </c>
+      <c r="C342">
+        <v>2026</v>
+      </c>
+      <c r="D342" s="0">
+        <v>16</v>
+      </c>
+      <c r="E342" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F342" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B343" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C343">
+        <v>2026</v>
+      </c>
+      <c r="D343" s="0">
+        <v>16</v>
+      </c>
+      <c r="E343" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F343" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B344" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C344">
+        <v>2026</v>
+      </c>
+      <c r="D344" s="0">
+        <v>16</v>
+      </c>
+      <c r="E344" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F344" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B345" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C345">
+        <v>2026</v>
+      </c>
+      <c r="D345" s="0">
+        <v>16</v>
+      </c>
+      <c r="E345" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F345" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B346" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C346">
+        <v>2026</v>
+      </c>
+      <c r="D346" s="0">
+        <v>16</v>
+      </c>
+      <c r="E346" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F346" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B347" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C347">
+        <v>2026</v>
+      </c>
+      <c r="D347" s="0">
+        <v>16</v>
+      </c>
+      <c r="E347" s="10" t="s">
+        <v>1067</v>
+      </c>
+      <c r="F347" s="10" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B348" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C348">
+        <v>2026</v>
+      </c>
+      <c r="D348" s="0">
+        <v>16</v>
+      </c>
+      <c r="E348" s="10" t="s">
+        <v>1067</v>
+      </c>
+      <c r="F348" s="10" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B349" t="s">
+        <v>1041</v>
+      </c>
+      <c r="C349">
+        <v>2026</v>
+      </c>
+      <c r="D349" s="0">
+        <v>16</v>
+      </c>
+      <c r="E349" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F349" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B350" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C350">
+        <v>2026</v>
+      </c>
+      <c r="D350" s="0">
+        <v>16</v>
+      </c>
+      <c r="E350" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F350" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B351" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C351">
+        <v>2026</v>
+      </c>
+      <c r="D351" s="0">
+        <v>16</v>
+      </c>
+      <c r="E351" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F351" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B352" t="s">
+        <v>1056</v>
+      </c>
+      <c r="C352">
+        <v>2026</v>
+      </c>
+      <c r="D352" s="0">
+        <v>16</v>
+      </c>
+      <c r="E352" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F352" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B353" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C353">
+        <v>2026</v>
+      </c>
+      <c r="D353" s="0">
+        <v>16</v>
+      </c>
+      <c r="E353" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F353" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated stats after Bahrain
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -3238,6 +3238,9 @@
   </si>
   <si>
     <t>17-2</t>
+  </si>
+  <si>
+    <t>13-5</t>
   </si>
 </sst>
 </file>
@@ -11173,6 +11176,446 @@
         <v>106</v>
       </c>
     </row>
+    <row r="354">
+      <c r="A354" t="s">
+        <v>955</v>
+      </c>
+      <c r="B354" t="s">
+        <v>956</v>
+      </c>
+      <c r="C354">
+        <v>2026</v>
+      </c>
+      <c r="D354" s="0">
+        <v>17</v>
+      </c>
+      <c r="E354" s="10" t="s">
+        <v>577</v>
+      </c>
+      <c r="F354" s="10" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="s">
+        <v>960</v>
+      </c>
+      <c r="B355" t="s">
+        <v>961</v>
+      </c>
+      <c r="C355">
+        <v>2026</v>
+      </c>
+      <c r="D355" s="0">
+        <v>17</v>
+      </c>
+      <c r="E355" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="F355" s="10" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="s">
+        <v>965</v>
+      </c>
+      <c r="B356" t="s">
+        <v>966</v>
+      </c>
+      <c r="C356">
+        <v>2026</v>
+      </c>
+      <c r="D356" s="0">
+        <v>17</v>
+      </c>
+      <c r="E356" s="10" t="s">
+        <v>297</v>
+      </c>
+      <c r="F356" s="10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="s">
+        <v>970</v>
+      </c>
+      <c r="B357" t="s">
+        <v>971</v>
+      </c>
+      <c r="C357">
+        <v>2026</v>
+      </c>
+      <c r="D357" s="0">
+        <v>17</v>
+      </c>
+      <c r="E357" s="10" t="s">
+        <v>497</v>
+      </c>
+      <c r="F357" s="10" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="s">
+        <v>975</v>
+      </c>
+      <c r="B358" t="s">
+        <v>976</v>
+      </c>
+      <c r="C358">
+        <v>2026</v>
+      </c>
+      <c r="D358" s="0">
+        <v>17</v>
+      </c>
+      <c r="E358" s="10" t="s">
+        <v>1075</v>
+      </c>
+      <c r="F358" s="10" t="s">
+        <v>1075</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="s">
+        <v>980</v>
+      </c>
+      <c r="B359" t="s">
+        <v>981</v>
+      </c>
+      <c r="C359">
+        <v>2026</v>
+      </c>
+      <c r="D359" s="0">
+        <v>17</v>
+      </c>
+      <c r="E359" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F359" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="s">
+        <v>985</v>
+      </c>
+      <c r="B360" t="s">
+        <v>986</v>
+      </c>
+      <c r="C360">
+        <v>2026</v>
+      </c>
+      <c r="D360" s="0">
+        <v>17</v>
+      </c>
+      <c r="E360" s="10" t="s">
+        <v>481</v>
+      </c>
+      <c r="F360" s="10" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="s">
+        <v>990</v>
+      </c>
+      <c r="B361" t="s">
+        <v>991</v>
+      </c>
+      <c r="C361">
+        <v>2026</v>
+      </c>
+      <c r="D361" s="0">
+        <v>17</v>
+      </c>
+      <c r="E361" s="10" t="s">
+        <v>481</v>
+      </c>
+      <c r="F361" s="10" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="s">
+        <v>995</v>
+      </c>
+      <c r="B362" t="s">
+        <v>996</v>
+      </c>
+      <c r="C362">
+        <v>2026</v>
+      </c>
+      <c r="D362" s="0">
+        <v>17</v>
+      </c>
+      <c r="E362" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F362" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B363" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C363">
+        <v>2026</v>
+      </c>
+      <c r="D363" s="0">
+        <v>17</v>
+      </c>
+      <c r="E363" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F363" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B364" t="s">
+        <v>1006</v>
+      </c>
+      <c r="C364">
+        <v>2026</v>
+      </c>
+      <c r="D364" s="0">
+        <v>17</v>
+      </c>
+      <c r="E364" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F364" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B365" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C365">
+        <v>2026</v>
+      </c>
+      <c r="D365" s="0">
+        <v>17</v>
+      </c>
+      <c r="E365" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F365" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B366" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C366">
+        <v>2026</v>
+      </c>
+      <c r="D366" s="0">
+        <v>17</v>
+      </c>
+      <c r="E366" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F366" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B367" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C367">
+        <v>2026</v>
+      </c>
+      <c r="D367" s="0">
+        <v>17</v>
+      </c>
+      <c r="E367" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F367" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B368" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C368">
+        <v>2026</v>
+      </c>
+      <c r="D368" s="0">
+        <v>17</v>
+      </c>
+      <c r="E368" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F368" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B369" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C369">
+        <v>2026</v>
+      </c>
+      <c r="D369" s="0">
+        <v>17</v>
+      </c>
+      <c r="E369" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F369" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B370" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C370">
+        <v>2026</v>
+      </c>
+      <c r="D370" s="0">
+        <v>17</v>
+      </c>
+      <c r="E370" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F370" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B371" t="s">
+        <v>1041</v>
+      </c>
+      <c r="C371">
+        <v>2026</v>
+      </c>
+      <c r="D371" s="0">
+        <v>17</v>
+      </c>
+      <c r="E371" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F371" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B372" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C372">
+        <v>2026</v>
+      </c>
+      <c r="D372" s="0">
+        <v>17</v>
+      </c>
+      <c r="E372" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F372" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B373" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C373">
+        <v>2026</v>
+      </c>
+      <c r="D373" s="0">
+        <v>17</v>
+      </c>
+      <c r="E373" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F373" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B374" t="s">
+        <v>1056</v>
+      </c>
+      <c r="C374">
+        <v>2026</v>
+      </c>
+      <c r="D374" s="0">
+        <v>17</v>
+      </c>
+      <c r="E374" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F374" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B375" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C375">
+        <v>2026</v>
+      </c>
+      <c r="D375" s="0">
+        <v>17</v>
+      </c>
+      <c r="E375" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F375" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Stats and team ahead of Austin, USA
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -3241,6 +3241,12 @@
   </si>
   <si>
     <t>13-5</t>
+  </si>
+  <si>
+    <t>15-8</t>
+  </si>
+  <si>
+    <t>15-1</t>
   </si>
 </sst>
 </file>
@@ -11189,11 +11195,14 @@
       <c r="D354" s="0">
         <v>17</v>
       </c>
-      <c r="E354" s="10" t="s">
-        <v>577</v>
+      <c r="E354" s="0" t="s">
+        <v>297</v>
       </c>
       <c r="F354" s="10" t="s">
         <v>577</v>
+      </c>
+      <c r="H354" s="0" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="355">
@@ -11209,11 +11218,14 @@
       <c r="D355" s="0">
         <v>17</v>
       </c>
-      <c r="E355" s="10" t="s">
-        <v>237</v>
+      <c r="E355" s="0" t="s">
+        <v>305</v>
       </c>
       <c r="F355" s="10" t="s">
         <v>237</v>
+      </c>
+      <c r="H355" s="0" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="356">
@@ -11229,11 +11241,14 @@
       <c r="D356" s="0">
         <v>17</v>
       </c>
-      <c r="E356" s="10" t="s">
-        <v>297</v>
+      <c r="E356" s="0" t="s">
+        <v>763</v>
       </c>
       <c r="F356" s="10" t="s">
         <v>297</v>
+      </c>
+      <c r="H356" s="0" t="s">
+        <v>763</v>
       </c>
     </row>
     <row r="357">
@@ -11249,11 +11264,14 @@
       <c r="D357" s="0">
         <v>17</v>
       </c>
-      <c r="E357" s="10" t="s">
-        <v>497</v>
+      <c r="E357" s="0" t="s">
+        <v>481</v>
       </c>
       <c r="F357" s="10" t="s">
         <v>497</v>
+      </c>
+      <c r="H357" s="0" t="s">
+        <v>481</v>
       </c>
     </row>
     <row r="358">
@@ -11269,11 +11287,14 @@
       <c r="D358" s="0">
         <v>17</v>
       </c>
-      <c r="E358" s="10" t="s">
-        <v>1075</v>
+      <c r="E358" s="0" t="s">
+        <v>1076</v>
       </c>
       <c r="F358" s="10" t="s">
         <v>1075</v>
+      </c>
+      <c r="H358" s="0" t="s">
+        <v>1076</v>
       </c>
     </row>
     <row r="359">
@@ -11289,11 +11310,14 @@
       <c r="D359" s="0">
         <v>17</v>
       </c>
-      <c r="E359" s="10" t="s">
-        <v>11</v>
+      <c r="E359" s="0" t="s">
+        <v>409</v>
       </c>
       <c r="F359" s="10" t="s">
         <v>11</v>
+      </c>
+      <c r="H359" s="0" t="s">
+        <v>409</v>
       </c>
     </row>
     <row r="360">
@@ -11309,11 +11333,14 @@
       <c r="D360" s="0">
         <v>17</v>
       </c>
-      <c r="E360" s="10" t="s">
-        <v>481</v>
+      <c r="E360" s="0" t="s">
+        <v>297</v>
       </c>
       <c r="F360" s="10" t="s">
         <v>481</v>
+      </c>
+      <c r="H360" s="0" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="361">
@@ -11329,11 +11356,14 @@
       <c r="D361" s="0">
         <v>17</v>
       </c>
-      <c r="E361" s="10" t="s">
-        <v>481</v>
+      <c r="E361" s="0" t="s">
+        <v>485</v>
       </c>
       <c r="F361" s="10" t="s">
         <v>481</v>
+      </c>
+      <c r="H361" s="0" t="s">
+        <v>485</v>
       </c>
     </row>
     <row r="362">
@@ -11349,11 +11379,14 @@
       <c r="D362" s="0">
         <v>17</v>
       </c>
-      <c r="E362" s="10" t="s">
-        <v>56</v>
+      <c r="E362" s="0" t="s">
+        <v>71</v>
       </c>
       <c r="F362" s="10" t="s">
         <v>56</v>
+      </c>
+      <c r="H362" s="0" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="363">
@@ -11369,11 +11402,14 @@
       <c r="D363" s="0">
         <v>17</v>
       </c>
-      <c r="E363" s="10" t="s">
-        <v>56</v>
+      <c r="E363" s="0" t="s">
+        <v>71</v>
       </c>
       <c r="F363" s="10" t="s">
         <v>56</v>
+      </c>
+      <c r="H363" s="0" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="364">
@@ -11389,11 +11425,14 @@
       <c r="D364" s="0">
         <v>17</v>
       </c>
-      <c r="E364" s="10" t="s">
-        <v>56</v>
+      <c r="E364" s="0" t="s">
+        <v>106</v>
       </c>
       <c r="F364" s="10" t="s">
         <v>56</v>
+      </c>
+      <c r="H364" s="0" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="365">
@@ -11409,11 +11448,14 @@
       <c r="D365" s="0">
         <v>17</v>
       </c>
-      <c r="E365" s="10" t="s">
-        <v>56</v>
+      <c r="E365" s="0" t="s">
+        <v>106</v>
       </c>
       <c r="F365" s="10" t="s">
         <v>56</v>
+      </c>
+      <c r="H365" s="0" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="366">
@@ -11429,11 +11471,14 @@
       <c r="D366" s="0">
         <v>17</v>
       </c>
-      <c r="E366" s="10" t="s">
-        <v>56</v>
+      <c r="E366" s="0" t="s">
+        <v>106</v>
       </c>
       <c r="F366" s="10" t="s">
         <v>56</v>
+      </c>
+      <c r="H366" s="0" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="367">
@@ -11449,11 +11494,14 @@
       <c r="D367" s="0">
         <v>17</v>
       </c>
-      <c r="E367" s="10" t="s">
-        <v>56</v>
+      <c r="E367" s="0" t="s">
+        <v>241</v>
       </c>
       <c r="F367" s="10" t="s">
         <v>56</v>
+      </c>
+      <c r="H367" s="0" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="368">
@@ -11469,11 +11517,14 @@
       <c r="D368" s="0">
         <v>17</v>
       </c>
-      <c r="E368" s="10" t="s">
-        <v>56</v>
+      <c r="E368" s="0" t="s">
+        <v>193</v>
       </c>
       <c r="F368" s="10" t="s">
         <v>56</v>
+      </c>
+      <c r="H368" s="0" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="369">
@@ -11489,11 +11540,14 @@
       <c r="D369" s="0">
         <v>17</v>
       </c>
-      <c r="E369" s="10" t="s">
-        <v>56</v>
+      <c r="E369" s="0" t="s">
+        <v>193</v>
       </c>
       <c r="F369" s="10" t="s">
         <v>56</v>
+      </c>
+      <c r="H369" s="0" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="370">
@@ -11509,11 +11563,14 @@
       <c r="D370" s="0">
         <v>17</v>
       </c>
-      <c r="E370" s="10" t="s">
-        <v>56</v>
+      <c r="E370" s="0" t="s">
+        <v>106</v>
       </c>
       <c r="F370" s="10" t="s">
         <v>56</v>
+      </c>
+      <c r="H370" s="0" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="371">
@@ -11529,11 +11586,14 @@
       <c r="D371" s="0">
         <v>17</v>
       </c>
-      <c r="E371" s="10" t="s">
-        <v>56</v>
+      <c r="E371" s="0" t="s">
+        <v>106</v>
       </c>
       <c r="F371" s="10" t="s">
         <v>56</v>
+      </c>
+      <c r="H371" s="0" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="372">
@@ -11549,11 +11609,14 @@
       <c r="D372" s="0">
         <v>17</v>
       </c>
-      <c r="E372" s="10" t="s">
-        <v>56</v>
+      <c r="E372" s="0" t="s">
+        <v>897</v>
       </c>
       <c r="F372" s="10" t="s">
         <v>56</v>
+      </c>
+      <c r="H372" s="0" t="s">
+        <v>897</v>
       </c>
     </row>
     <row r="373">
@@ -11569,11 +11632,14 @@
       <c r="D373" s="0">
         <v>17</v>
       </c>
-      <c r="E373" s="10" t="s">
-        <v>56</v>
+      <c r="E373" s="0" t="s">
+        <v>106</v>
       </c>
       <c r="F373" s="10" t="s">
         <v>56</v>
+      </c>
+      <c r="H373" s="0" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="374">
@@ -11589,11 +11655,14 @@
       <c r="D374" s="0">
         <v>17</v>
       </c>
-      <c r="E374" s="10" t="s">
-        <v>106</v>
+      <c r="E374" s="0" t="s">
+        <v>345</v>
       </c>
       <c r="F374" s="10" t="s">
         <v>106</v>
+      </c>
+      <c r="H374" s="0" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="375">
@@ -11609,10 +11678,453 @@
       <c r="D375" s="0">
         <v>17</v>
       </c>
-      <c r="E375" s="10" t="s">
+      <c r="E375" s="0" t="s">
+        <v>345</v>
+      </c>
+      <c r="F375" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="F375" s="10" t="s">
+      <c r="H375" s="0" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="s">
+        <v>955</v>
+      </c>
+      <c r="B376" t="s">
+        <v>956</v>
+      </c>
+      <c r="C376">
+        <v>2026</v>
+      </c>
+      <c r="D376" s="0">
+        <v>18</v>
+      </c>
+      <c r="E376" s="10" t="s">
+        <v>1077</v>
+      </c>
+      <c r="F376" s="10" t="s">
+        <v>1077</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="s">
+        <v>960</v>
+      </c>
+      <c r="B377" t="s">
+        <v>961</v>
+      </c>
+      <c r="C377">
+        <v>2026</v>
+      </c>
+      <c r="D377" s="0">
+        <v>18</v>
+      </c>
+      <c r="E377" s="10" t="s">
+        <v>1071</v>
+      </c>
+      <c r="F377" s="10" t="s">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="s">
+        <v>965</v>
+      </c>
+      <c r="B378" t="s">
+        <v>966</v>
+      </c>
+      <c r="C378">
+        <v>2026</v>
+      </c>
+      <c r="D378" s="0">
+        <v>18</v>
+      </c>
+      <c r="E378" s="10" t="s">
+        <v>477</v>
+      </c>
+      <c r="F378" s="10" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="s">
+        <v>970</v>
+      </c>
+      <c r="B379" t="s">
+        <v>971</v>
+      </c>
+      <c r="C379">
+        <v>2026</v>
+      </c>
+      <c r="D379" s="0">
+        <v>18</v>
+      </c>
+      <c r="E379" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F379" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="s">
+        <v>975</v>
+      </c>
+      <c r="B380" t="s">
+        <v>976</v>
+      </c>
+      <c r="C380">
+        <v>2026</v>
+      </c>
+      <c r="D380" s="0">
+        <v>18</v>
+      </c>
+      <c r="E380" s="10" t="s">
+        <v>1075</v>
+      </c>
+      <c r="F380" s="10" t="s">
+        <v>1075</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="s">
+        <v>980</v>
+      </c>
+      <c r="B381" t="s">
+        <v>981</v>
+      </c>
+      <c r="C381">
+        <v>2026</v>
+      </c>
+      <c r="D381" s="0">
+        <v>18</v>
+      </c>
+      <c r="E381" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="F381" s="10" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="s">
+        <v>985</v>
+      </c>
+      <c r="B382" t="s">
+        <v>986</v>
+      </c>
+      <c r="C382">
+        <v>2026</v>
+      </c>
+      <c r="D382" s="0">
+        <v>18</v>
+      </c>
+      <c r="E382" s="10" t="s">
+        <v>477</v>
+      </c>
+      <c r="F382" s="10" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="s">
+        <v>990</v>
+      </c>
+      <c r="B383" t="s">
+        <v>991</v>
+      </c>
+      <c r="C383">
+        <v>2026</v>
+      </c>
+      <c r="D383" s="0">
+        <v>18</v>
+      </c>
+      <c r="E383" s="10" t="s">
+        <v>477</v>
+      </c>
+      <c r="F383" s="10" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="s">
+        <v>995</v>
+      </c>
+      <c r="B384" t="s">
+        <v>996</v>
+      </c>
+      <c r="C384">
+        <v>2026</v>
+      </c>
+      <c r="D384" s="0">
+        <v>18</v>
+      </c>
+      <c r="E384" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F384" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B385" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C385">
+        <v>2026</v>
+      </c>
+      <c r="D385" s="0">
+        <v>18</v>
+      </c>
+      <c r="E385" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F385" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B386" t="s">
+        <v>1006</v>
+      </c>
+      <c r="C386">
+        <v>2026</v>
+      </c>
+      <c r="D386" s="0">
+        <v>18</v>
+      </c>
+      <c r="E386" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F386" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B387" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C387">
+        <v>2026</v>
+      </c>
+      <c r="D387" s="0">
+        <v>18</v>
+      </c>
+      <c r="E387" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F387" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B388" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C388">
+        <v>2026</v>
+      </c>
+      <c r="D388" s="0">
+        <v>18</v>
+      </c>
+      <c r="E388" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F388" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B389" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C389">
+        <v>2026</v>
+      </c>
+      <c r="D389" s="0">
+        <v>18</v>
+      </c>
+      <c r="E389" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F389" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B390" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C390">
+        <v>2026</v>
+      </c>
+      <c r="D390" s="0">
+        <v>18</v>
+      </c>
+      <c r="E390" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F390" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B391" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C391">
+        <v>2026</v>
+      </c>
+      <c r="D391" s="0">
+        <v>18</v>
+      </c>
+      <c r="E391" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F391" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B392" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C392">
+        <v>2026</v>
+      </c>
+      <c r="D392" s="0">
+        <v>18</v>
+      </c>
+      <c r="E392" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F392" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B393" t="s">
+        <v>1041</v>
+      </c>
+      <c r="C393">
+        <v>2026</v>
+      </c>
+      <c r="D393" s="0">
+        <v>18</v>
+      </c>
+      <c r="E393" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F393" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B394" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C394">
+        <v>2026</v>
+      </c>
+      <c r="D394" s="0">
+        <v>18</v>
+      </c>
+      <c r="E394" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F394" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B395" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C395">
+        <v>2026</v>
+      </c>
+      <c r="D395" s="0">
+        <v>18</v>
+      </c>
+      <c r="E395" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F395" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B396" t="s">
+        <v>1056</v>
+      </c>
+      <c r="C396">
+        <v>2026</v>
+      </c>
+      <c r="D396" s="0">
+        <v>18</v>
+      </c>
+      <c r="E396" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F396" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B397" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C397">
+        <v>2026</v>
+      </c>
+      <c r="D397" s="0">
+        <v>18</v>
+      </c>
+      <c r="E397" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F397" s="10" t="s">
         <v>106</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated after America before Mexico
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -3247,6 +3247,12 @@
   </si>
   <si>
     <t>15-1</t>
+  </si>
+  <si>
+    <t>8-5</t>
+  </si>
+  <si>
+    <t>45-1</t>
   </si>
 </sst>
 </file>
@@ -12128,6 +12134,446 @@
         <v>106</v>
       </c>
     </row>
+    <row r="398">
+      <c r="A398" t="s">
+        <v>955</v>
+      </c>
+      <c r="B398" t="s">
+        <v>956</v>
+      </c>
+      <c r="C398">
+        <v>2026</v>
+      </c>
+      <c r="D398" s="0">
+        <v>19</v>
+      </c>
+      <c r="E398" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="F398" s="10" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="s">
+        <v>960</v>
+      </c>
+      <c r="B399" t="s">
+        <v>961</v>
+      </c>
+      <c r="C399">
+        <v>2026</v>
+      </c>
+      <c r="D399" s="0">
+        <v>19</v>
+      </c>
+      <c r="E399" s="10" t="s">
+        <v>1079</v>
+      </c>
+      <c r="F399" s="10" t="s">
+        <v>1079</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="s">
+        <v>965</v>
+      </c>
+      <c r="B400" t="s">
+        <v>966</v>
+      </c>
+      <c r="C400">
+        <v>2026</v>
+      </c>
+      <c r="D400" s="0">
+        <v>19</v>
+      </c>
+      <c r="E400" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="F400" s="10" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="s">
+        <v>970</v>
+      </c>
+      <c r="B401" t="s">
+        <v>971</v>
+      </c>
+      <c r="C401">
+        <v>2026</v>
+      </c>
+      <c r="D401" s="0">
+        <v>19</v>
+      </c>
+      <c r="E401" s="10" t="s">
+        <v>1076</v>
+      </c>
+      <c r="F401" s="10" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="s">
+        <v>975</v>
+      </c>
+      <c r="B402" t="s">
+        <v>976</v>
+      </c>
+      <c r="C402">
+        <v>2026</v>
+      </c>
+      <c r="D402" s="0">
+        <v>19</v>
+      </c>
+      <c r="E402" s="10" t="s">
+        <v>1078</v>
+      </c>
+      <c r="F402" s="10" t="s">
+        <v>1078</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="s">
+        <v>980</v>
+      </c>
+      <c r="B403" t="s">
+        <v>981</v>
+      </c>
+      <c r="C403">
+        <v>2026</v>
+      </c>
+      <c r="D403" s="0">
+        <v>19</v>
+      </c>
+      <c r="E403" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="F403" s="10" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="s">
+        <v>985</v>
+      </c>
+      <c r="B404" t="s">
+        <v>986</v>
+      </c>
+      <c r="C404">
+        <v>2026</v>
+      </c>
+      <c r="D404" s="0">
+        <v>19</v>
+      </c>
+      <c r="E404" s="10" t="s">
+        <v>305</v>
+      </c>
+      <c r="F404" s="10" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="s">
+        <v>990</v>
+      </c>
+      <c r="B405" t="s">
+        <v>991</v>
+      </c>
+      <c r="C405">
+        <v>2026</v>
+      </c>
+      <c r="D405" s="0">
+        <v>19</v>
+      </c>
+      <c r="E405" s="10" t="s">
+        <v>297</v>
+      </c>
+      <c r="F405" s="10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="s">
+        <v>995</v>
+      </c>
+      <c r="B406" t="s">
+        <v>996</v>
+      </c>
+      <c r="C406">
+        <v>2026</v>
+      </c>
+      <c r="D406" s="0">
+        <v>19</v>
+      </c>
+      <c r="E406" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F406" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B407" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C407">
+        <v>2026</v>
+      </c>
+      <c r="D407" s="0">
+        <v>19</v>
+      </c>
+      <c r="E407" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F407" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B408" t="s">
+        <v>1006</v>
+      </c>
+      <c r="C408">
+        <v>2026</v>
+      </c>
+      <c r="D408" s="0">
+        <v>19</v>
+      </c>
+      <c r="E408" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F408" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B409" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C409">
+        <v>2026</v>
+      </c>
+      <c r="D409" s="0">
+        <v>19</v>
+      </c>
+      <c r="E409" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F409" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B410" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C410">
+        <v>2026</v>
+      </c>
+      <c r="D410" s="0">
+        <v>19</v>
+      </c>
+      <c r="E410" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F410" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B411" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C411">
+        <v>2026</v>
+      </c>
+      <c r="D411" s="0">
+        <v>19</v>
+      </c>
+      <c r="E411" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F411" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B412" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C412">
+        <v>2026</v>
+      </c>
+      <c r="D412" s="0">
+        <v>19</v>
+      </c>
+      <c r="E412" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F412" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B413" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C413">
+        <v>2026</v>
+      </c>
+      <c r="D413" s="0">
+        <v>19</v>
+      </c>
+      <c r="E413" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F413" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B414" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C414">
+        <v>2026</v>
+      </c>
+      <c r="D414" s="0">
+        <v>19</v>
+      </c>
+      <c r="E414" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F414" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B415" t="s">
+        <v>1041</v>
+      </c>
+      <c r="C415">
+        <v>2026</v>
+      </c>
+      <c r="D415" s="0">
+        <v>19</v>
+      </c>
+      <c r="E415" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F415" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B416" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C416">
+        <v>2026</v>
+      </c>
+      <c r="D416" s="0">
+        <v>19</v>
+      </c>
+      <c r="E416" s="10" t="s">
+        <v>1067</v>
+      </c>
+      <c r="F416" s="10" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B417" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C417">
+        <v>2026</v>
+      </c>
+      <c r="D417" s="0">
+        <v>19</v>
+      </c>
+      <c r="E417" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F417" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B418" t="s">
+        <v>1056</v>
+      </c>
+      <c r="C418">
+        <v>2026</v>
+      </c>
+      <c r="D418" s="0">
+        <v>19</v>
+      </c>
+      <c r="E418" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F418" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B419" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C419">
+        <v>2026</v>
+      </c>
+      <c r="D419" s="0">
+        <v>19</v>
+      </c>
+      <c r="E419" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F419" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 2026 Mexico (R19) post-FP2 betting odds
Updates Odds and Odds_Post_FP2 for 2026 race 19 only; no other row or
column changed.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -3253,6 +3253,12 @@
   </si>
   <si>
     <t>45-1</t>
+  </si>
+  <si>
+    <t>3-1</t>
+  </si>
+  <si>
+    <t>75-1</t>
   </si>
 </sst>
 </file>
@@ -12147,11 +12153,14 @@
       <c r="D398" s="0">
         <v>19</v>
       </c>
-      <c r="E398" s="10" t="s">
-        <v>213</v>
+      <c r="E398" s="0" t="s">
+        <v>11</v>
       </c>
       <c r="F398" s="10" t="s">
         <v>213</v>
+      </c>
+      <c r="H398" s="0" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="399">
@@ -12167,11 +12176,14 @@
       <c r="D399" s="0">
         <v>19</v>
       </c>
-      <c r="E399" s="10" t="s">
-        <v>1079</v>
+      <c r="E399" s="0" t="s">
+        <v>675</v>
       </c>
       <c r="F399" s="10" t="s">
         <v>1079</v>
+      </c>
+      <c r="H399" s="0" t="s">
+        <v>675</v>
       </c>
     </row>
     <row r="400">
@@ -12187,11 +12199,14 @@
       <c r="D400" s="0">
         <v>19</v>
       </c>
-      <c r="E400" s="10" t="s">
-        <v>413</v>
+      <c r="E400" s="0" t="s">
+        <v>237</v>
       </c>
       <c r="F400" s="10" t="s">
         <v>413</v>
+      </c>
+      <c r="H400" s="0" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="401">
@@ -12207,11 +12222,14 @@
       <c r="D401" s="0">
         <v>19</v>
       </c>
-      <c r="E401" s="10" t="s">
-        <v>1076</v>
+      <c r="E401" s="0" t="s">
+        <v>397</v>
       </c>
       <c r="F401" s="10" t="s">
         <v>1076</v>
+      </c>
+      <c r="H401" s="0" t="s">
+        <v>397</v>
       </c>
     </row>
     <row r="402">
@@ -12227,11 +12245,14 @@
       <c r="D402" s="0">
         <v>19</v>
       </c>
-      <c r="E402" s="10" t="s">
-        <v>1078</v>
+      <c r="E402" s="0" t="s">
+        <v>1080</v>
       </c>
       <c r="F402" s="10" t="s">
         <v>1078</v>
+      </c>
+      <c r="H402" s="0" t="s">
+        <v>1080</v>
       </c>
     </row>
     <row r="403">
@@ -12247,11 +12268,14 @@
       <c r="D403" s="0">
         <v>19</v>
       </c>
-      <c r="E403" s="10" t="s">
-        <v>233</v>
+      <c r="E403" s="0" t="s">
+        <v>1081</v>
       </c>
       <c r="F403" s="10" t="s">
         <v>233</v>
+      </c>
+      <c r="H403" s="0" t="s">
+        <v>1081</v>
       </c>
     </row>
     <row r="404">
@@ -12267,11 +12291,14 @@
       <c r="D404" s="0">
         <v>19</v>
       </c>
-      <c r="E404" s="10" t="s">
-        <v>305</v>
+      <c r="E404" s="0" t="s">
+        <v>11</v>
       </c>
       <c r="F404" s="10" t="s">
         <v>305</v>
+      </c>
+      <c r="H404" s="0" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="405">
@@ -12287,11 +12314,14 @@
       <c r="D405" s="0">
         <v>19</v>
       </c>
-      <c r="E405" s="10" t="s">
-        <v>297</v>
+      <c r="E405" s="0" t="s">
+        <v>149</v>
       </c>
       <c r="F405" s="10" t="s">
         <v>297</v>
+      </c>
+      <c r="H405" s="0" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="406">
@@ -12307,11 +12337,14 @@
       <c r="D406" s="0">
         <v>19</v>
       </c>
-      <c r="E406" s="10" t="s">
-        <v>106</v>
+      <c r="E406" s="0" t="s">
+        <v>71</v>
       </c>
       <c r="F406" s="10" t="s">
         <v>106</v>
+      </c>
+      <c r="H406" s="0" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="407">
@@ -12327,11 +12360,14 @@
       <c r="D407" s="0">
         <v>19</v>
       </c>
-      <c r="E407" s="10" t="s">
-        <v>106</v>
+      <c r="E407" s="0" t="s">
+        <v>71</v>
       </c>
       <c r="F407" s="10" t="s">
         <v>106</v>
+      </c>
+      <c r="H407" s="0" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="408">
@@ -12347,10 +12383,13 @@
       <c r="D408" s="0">
         <v>19</v>
       </c>
-      <c r="E408" s="10" t="s">
+      <c r="E408" s="0" t="s">
         <v>56</v>
       </c>
       <c r="F408" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H408" s="0" t="s">
         <v>56</v>
       </c>
     </row>
@@ -12367,11 +12406,14 @@
       <c r="D409" s="0">
         <v>19</v>
       </c>
-      <c r="E409" s="10" t="s">
-        <v>66</v>
+      <c r="E409" s="0" t="s">
+        <v>56</v>
       </c>
       <c r="F409" s="10" t="s">
         <v>66</v>
+      </c>
+      <c r="H409" s="0" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="410">
@@ -12387,11 +12429,14 @@
       <c r="D410" s="0">
         <v>19</v>
       </c>
-      <c r="E410" s="10" t="s">
-        <v>106</v>
+      <c r="E410" s="0" t="s">
+        <v>169</v>
       </c>
       <c r="F410" s="10" t="s">
         <v>106</v>
+      </c>
+      <c r="H410" s="0" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="411">
@@ -12407,11 +12452,14 @@
       <c r="D411" s="0">
         <v>19</v>
       </c>
-      <c r="E411" s="10" t="s">
-        <v>106</v>
+      <c r="E411" s="0" t="s">
+        <v>241</v>
       </c>
       <c r="F411" s="10" t="s">
         <v>106</v>
+      </c>
+      <c r="H411" s="0" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="412">
@@ -12427,11 +12475,14 @@
       <c r="D412" s="0">
         <v>19</v>
       </c>
-      <c r="E412" s="10" t="s">
-        <v>106</v>
+      <c r="E412" s="0" t="s">
+        <v>193</v>
       </c>
       <c r="F412" s="10" t="s">
         <v>106</v>
+      </c>
+      <c r="H412" s="0" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="413">
@@ -12447,11 +12498,14 @@
       <c r="D413" s="0">
         <v>19</v>
       </c>
-      <c r="E413" s="10" t="s">
-        <v>106</v>
+      <c r="E413" s="0" t="s">
+        <v>193</v>
       </c>
       <c r="F413" s="10" t="s">
         <v>106</v>
+      </c>
+      <c r="H413" s="0" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="414">
@@ -12467,11 +12521,14 @@
       <c r="D414" s="0">
         <v>19</v>
       </c>
-      <c r="E414" s="10" t="s">
-        <v>106</v>
+      <c r="E414" s="0" t="s">
+        <v>193</v>
       </c>
       <c r="F414" s="10" t="s">
         <v>106</v>
+      </c>
+      <c r="H414" s="0" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="415">
@@ -12487,11 +12544,14 @@
       <c r="D415" s="0">
         <v>19</v>
       </c>
-      <c r="E415" s="10" t="s">
-        <v>51</v>
+      <c r="E415" s="0" t="s">
+        <v>193</v>
       </c>
       <c r="F415" s="10" t="s">
         <v>51</v>
+      </c>
+      <c r="H415" s="0" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="416">
@@ -12507,10 +12567,13 @@
       <c r="D416" s="0">
         <v>19</v>
       </c>
-      <c r="E416" s="10" t="s">
+      <c r="E416" s="0" t="s">
         <v>1067</v>
       </c>
       <c r="F416" s="10" t="s">
+        <v>1067</v>
+      </c>
+      <c r="H416" s="0" t="s">
         <v>1067</v>
       </c>
     </row>
@@ -12527,11 +12590,14 @@
       <c r="D417" s="0">
         <v>19</v>
       </c>
-      <c r="E417" s="10" t="s">
-        <v>51</v>
+      <c r="E417" s="0" t="s">
+        <v>193</v>
       </c>
       <c r="F417" s="10" t="s">
         <v>51</v>
+      </c>
+      <c r="H417" s="0" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="418">
@@ -12547,11 +12613,14 @@
       <c r="D418" s="0">
         <v>19</v>
       </c>
-      <c r="E418" s="10" t="s">
-        <v>106</v>
+      <c r="E418" s="0" t="s">
+        <v>709</v>
       </c>
       <c r="F418" s="10" t="s">
         <v>106</v>
+      </c>
+      <c r="H418" s="0" t="s">
+        <v>709</v>
       </c>
     </row>
     <row r="419">
@@ -12567,11 +12636,14 @@
       <c r="D419" s="0">
         <v>19</v>
       </c>
-      <c r="E419" s="10" t="s">
-        <v>106</v>
+      <c r="E419" s="0" t="s">
+        <v>709</v>
       </c>
       <c r="F419" s="10" t="s">
         <v>106</v>
+      </c>
+      <c r="H419" s="0" t="s">
+        <v>709</v>
       </c>
     </row>
   </sheetData>

</xml_diff>